<commit_message>
Hoja masiva: corregir los valores que Amazon rechazó en la 1ª subida
- Estado: Activado / En pausa (en vez de Habilitado / Pausado).
- Estrategia de pujas vacía (por defecto en campañas nuevas: solo reducir).
- El producto negativo (propia ficha) pasa a hacerse a mano: Amazon no
  aceptó 'Segmentación por productos negativa' como entidad.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8zFsXd31MYxmY7hRPcJU8
</commit_message>
<xml_diff>
--- a/resultados/bulk_2026-09-26.xlsx
+++ b/resultados/bulk_2026-09-26.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF52"/>
+  <dimension ref="A1:AF51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -690,17 +690,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Pausado</t>
+          <t>En pausa</t>
         </is>
       </c>
       <c r="P2" t="n">
         <v>7</v>
       </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>Pujas dinámicas: solo reducir</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -735,7 +730,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="R3" t="n">
@@ -770,7 +765,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -807,7 +802,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S5" t="n">
@@ -852,7 +847,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S6" t="n">
@@ -897,7 +892,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S7" t="n">
@@ -942,7 +937,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S8" t="n">
@@ -987,7 +982,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S9" t="n">
@@ -1032,7 +1027,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S10" t="n">
@@ -1077,7 +1072,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S11" t="n">
@@ -1122,7 +1117,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S12" t="n">
@@ -1167,7 +1162,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S13" t="n">
@@ -1212,7 +1207,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S14" t="n">
@@ -1257,7 +1252,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1299,7 +1294,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1341,7 +1336,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -1383,7 +1378,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -1425,7 +1420,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -1467,7 +1462,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
@@ -1509,7 +1504,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -1551,7 +1546,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -1603,17 +1598,12 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Pausado</t>
+          <t>En pausa</t>
         </is>
       </c>
       <c r="P23" t="n">
         <v>7</v>
       </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>Pujas dinámicas: solo reducir</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1648,7 +1638,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="R24" t="n">
@@ -1683,7 +1673,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -1720,7 +1710,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S26" t="n">
@@ -1760,7 +1750,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S27" t="n">
@@ -1800,7 +1790,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S28" t="n">
@@ -1840,7 +1830,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S29" t="n">
@@ -1860,7 +1850,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Segmentación por productos negativa</t>
+          <t>Campaña</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1870,23 +1860,31 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Pinza - Pruebas</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Pruebas - Competencia</t>
+          <t>Rejilla - Principal V2</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Rejilla - Principal V2</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>20260926</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Manual</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Habilitado</t>
-        </is>
-      </c>
-      <c r="AA30" t="inlineStr">
-        <is>
-          <t>asin="B0DCZS1NR6"</t>
-        </is>
+          <t>En pausa</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="31">
@@ -1897,7 +1895,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Campaña</t>
+          <t>Grupo de anuncios</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1910,33 +1908,23 @@
           <t>Rejilla - Principal V2</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Rejilla - Principal V2</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>20260926</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Manual</t>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Rejilla - Principal V2</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Rejilla - Principal V2</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Pausado</t>
-        </is>
-      </c>
-      <c r="P31" t="n">
-        <v>7</v>
-      </c>
-      <c r="X31" t="inlineStr">
-        <is>
-          <t>Pujas dinámicas: solo reducir</t>
-        </is>
+          <t>Activado</t>
+        </is>
+      </c>
+      <c r="R31" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="32">
@@ -1947,7 +1935,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Grupo de anuncios</t>
+          <t>Anuncio de producto</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1965,18 +1953,15 @@
           <t>Rejilla - Principal V2</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Rejilla - Principal V2</t>
-        </is>
-      </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Habilitado</t>
-        </is>
-      </c>
-      <c r="R32" t="n">
-        <v>0.4</v>
+          <t>Activado</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>5E-I8NY-S191</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1987,7 +1972,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Anuncio de producto</t>
+          <t>Palabra clave</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2007,12 +1992,20 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Habilitado</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>5E-I8NY-S191</t>
+          <t>Activado</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>soporte coche para teléfono móvil</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>Exacta</t>
         </is>
       </c>
     </row>
@@ -2044,15 +2037,15 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S34" t="n">
-        <v>0.48</v>
+        <v>0.24</v>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>soporte coche para teléfono móvil</t>
+          <t>soporte para móvil en coche</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
@@ -2089,20 +2082,20 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S35" t="n">
-        <v>0.24</v>
+        <v>0.48</v>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>soporte para móvil en coche</t>
+          <t>soporte teléfono para rejilla</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>Exacta</t>
+          <t>Frase</t>
         </is>
       </c>
     </row>
@@ -2134,15 +2127,15 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S36" t="n">
-        <v>0.48</v>
+        <v>0.38</v>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>soporte teléfono para rejilla</t>
+          <t>soporte móvil coche ventilación</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
@@ -2179,15 +2172,15 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S37" t="n">
-        <v>0.38</v>
+        <v>0.58</v>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>soporte móvil coche ventilación</t>
+          <t>soporte teléfono de rejilla ventilación</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
@@ -2224,15 +2217,15 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S38" t="n">
-        <v>0.58</v>
+        <v>0.41</v>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>soporte teléfono de rejilla ventilación</t>
+          <t>soporte teléfono rejilla coche con gancho</t>
         </is>
       </c>
       <c r="W38" t="inlineStr">
@@ -2269,15 +2262,15 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S39" t="n">
-        <v>0.41</v>
+        <v>0.4</v>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>soporte teléfono rejilla coche con gancho</t>
+          <t>rejilla móvil coche</t>
         </is>
       </c>
       <c r="W39" t="inlineStr">
@@ -2314,15 +2307,15 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S40" t="n">
-        <v>0.4</v>
+        <v>0.34</v>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>rejilla móvil coche</t>
+          <t>soporte rejilla móvil</t>
         </is>
       </c>
       <c r="W40" t="inlineStr">
@@ -2359,15 +2352,15 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S41" t="n">
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>soporte rejilla móvil</t>
+          <t>porta móvil de rejilla ventilación</t>
         </is>
       </c>
       <c r="W41" t="inlineStr">
@@ -2404,15 +2397,15 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="S42" t="n">
-        <v>0.32</v>
+        <v>0.25</v>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>porta móvil de rejilla ventilación</t>
+          <t>sujeta móvil de rejilla</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
@@ -2429,7 +2422,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Palabra clave</t>
+          <t>Palabra clave negativa</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2449,20 +2442,17 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Habilitado</t>
-        </is>
-      </c>
-      <c r="S43" t="n">
-        <v>0.25</v>
+          <t>Activado</t>
+        </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>sujeta móvil de rejilla</t>
+          <t>ventosa</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>Frase</t>
+          <t>Frase negativa</t>
         </is>
       </c>
     </row>
@@ -2494,12 +2484,12 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>ventosa</t>
+          <t>magnetico</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
@@ -2536,12 +2526,12 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>magnetico</t>
+          <t>iman</t>
         </is>
       </c>
       <c r="W45" t="inlineStr">
@@ -2578,12 +2568,12 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>iman</t>
+          <t>parabrisas</t>
         </is>
       </c>
       <c r="W46" t="inlineStr">
@@ -2620,12 +2610,12 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>parabrisas</t>
+          <t>moto</t>
         </is>
       </c>
       <c r="W47" t="inlineStr">
@@ -2662,12 +2652,12 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>moto</t>
+          <t>bicicleta</t>
         </is>
       </c>
       <c r="W48" t="inlineStr">
@@ -2704,12 +2694,12 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>bicicleta</t>
+          <t>cargador</t>
         </is>
       </c>
       <c r="W49" t="inlineStr">
@@ -2746,12 +2736,12 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>cargador</t>
+          <t>pinza</t>
         </is>
       </c>
       <c r="W50" t="inlineStr">
@@ -2788,57 +2778,15 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Habilitado</t>
+          <t>Activado</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>pinza</t>
+          <t>salpicadero</t>
         </is>
       </c>
       <c r="W51" t="inlineStr">
-        <is>
-          <t>Frase negativa</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Sponsored Products</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Palabra clave negativa</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Crear</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Rejilla - Principal V2</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Rejilla - Principal V2</t>
-        </is>
-      </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>Habilitado</t>
-        </is>
-      </c>
-      <c r="T52" t="inlineStr">
-        <is>
-          <t>salpicadero</t>
-        </is>
-      </c>
-      <c r="W52" t="inlineStr">
         <is>
           <t>Frase negativa</t>
         </is>

</xml_diff>